<commit_message>
add synthetic data for tests
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re5d45129421344ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R2d8da8a7542745fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rd84e0a01bbfd452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rae19b56dc84f4ea2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R2d7d436200244d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R067c356e7a8b4320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R9cf2fd93541b4db8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +50,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="44">
+  <x:fonts count="47">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -295,8 +296,25 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F1F1F"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -348,6 +366,16 @@
         <x:fgColor rgb="FF1F3864"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -369,7 +397,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="80">
+  <x:cellXfs count="102">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -588,10 +616,107 @@
     <x:xf numFmtId="0" fontId="43" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="44" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="44" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="45" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="45" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="45" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Κανονικό" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="4">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFE699"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF666666"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF2F2F2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -606,6 +731,37 @@
     <x:tableColumn id="6" name="Why it matters"/>
     <x:tableColumn id="7" name="Suggested Solution"/>
     <x:tableColumn id="8" name="Status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EventBusImplementationGroupsTable" displayName="EventBusImplementationGroupsTable" ref="A7:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="Group"/>
+    <x:tableColumn id="2" name="Workstream"/>
+    <x:tableColumn id="3" name="Tasks"/>
+    <x:tableColumn id="4" name="Safe parallel work"/>
+    <x:tableColumn id="5" name="Review sequence"/>
+    <x:tableColumn id="6" name="Start gate"/>
+    <x:tableColumn id="7" name="Group exit gate"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventBusReviewQueueTable" displayName="EventBusReviewQueueTable" ref="A23:H60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Task ID"/>
+    <x:tableColumn id="2" name="Group"/>
+    <x:tableColumn id="3" name="Phase"/>
+    <x:tableColumn id="4" name="Title"/>
+    <x:tableColumn id="5" name="Depends On"/>
+    <x:tableColumn id="6" name="Work Status"/>
+    <x:tableColumn id="7" name="Code Review"/>
+    <x:tableColumn id="8" name="Review commit / notes"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -911,6 +1067,14 @@
       <x:c r="D11"/>
       <x:c r="E11"/>
     </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="B12" t="str">
+        <x:v>Delivery rule: tasks share implementation groups, but each task remains its own code-review gate. Do not start the next task until the current task's code review is Approved. See Implementation Plan.</x:v>
+      </x:c>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+    </x:row>
     <x:row r="13" ht="15.75" customHeight="1">
       <x:c r="B13" s="3" t="s">
         <x:v>0</x:v>
@@ -2241,7 +2405,1389 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ef9a192fe44119"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4217b7315abd46c8"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Event Bus Implementation Groups &amp; Review Gates</x:v>
+      </x:c>
+      <x:c r="B1" s="81"/>
+      <x:c r="C1" s="81"/>
+      <x:c r="D1" s="81"/>
+      <x:c r="E1" s="81"/>
+      <x:c r="F1" s="81"/>
+      <x:c r="G1" s="81"/>
+      <x:c r="H1" s="81"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="85" t="str">
+        <x:v>Groups reduce context switching and expose safe parallel work. They do not combine reviews: implement one task, run focused tests, present the code/diff, wait for approval, then mark that task Approved and proceed. A group exits only when every task in it is Approved.</x:v>
+      </x:c>
+      <x:c r="B2" s="85"/>
+      <x:c r="C2" s="85"/>
+      <x:c r="D2" s="85"/>
+      <x:c r="E2" s="85"/>
+      <x:c r="F2" s="85"/>
+      <x:c r="G2" s="85"/>
+      <x:c r="H2" s="85"/>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="85"/>
+      <x:c r="B3" s="85"/>
+      <x:c r="C3" s="85"/>
+      <x:c r="D3" s="85"/>
+      <x:c r="E3" s="85"/>
+      <x:c r="F3" s="85"/>
+      <x:c r="G3" s="85"/>
+      <x:c r="H3" s="85"/>
+    </x:row>
+    <x:row r="5" ht="32" customHeight="1">
+      <x:c r="A5" s="91" t="str">
+        <x:v>Review workflow</x:v>
+      </x:c>
+      <x:c r="B5" s="91" t="str">
+        <x:v>1. Implement one task</x:v>
+      </x:c>
+      <x:c r="C5" s="91" t="str">
+        <x:v>2. Run focused tests</x:v>
+      </x:c>
+      <x:c r="D5" s="91" t="str">
+        <x:v>3. Present code review</x:v>
+      </x:c>
+      <x:c r="E5" s="91" t="str">
+        <x:v>4. Wait for approval</x:v>
+      </x:c>
+      <x:c r="F5" s="91" t="str">
+        <x:v>5. Commit/complete</x:v>
+      </x:c>
+      <x:c r="G5" s="91" t="str">
+        <x:v>6. Start next task</x:v>
+      </x:c>
+      <x:c r="H5" s="91" t="str">
+        <x:v>No batch approval</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="79" t="str">
+        <x:v>Group</x:v>
+      </x:c>
+      <x:c r="B7" s="79" t="str">
+        <x:v>Workstream</x:v>
+      </x:c>
+      <x:c r="C7" s="79" t="str">
+        <x:v>Tasks</x:v>
+      </x:c>
+      <x:c r="D7" s="79" t="str">
+        <x:v>Safe parallel work</x:v>
+      </x:c>
+      <x:c r="E7" s="79" t="str">
+        <x:v>Review sequence</x:v>
+      </x:c>
+      <x:c r="F7" s="79" t="str">
+        <x:v>Start gate</x:v>
+      </x:c>
+      <x:c r="G7" s="79" t="str">
+        <x:v>Group exit gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="50" customHeight="1">
+      <x:c r="A8" s="99" t="str">
+        <x:v>G00</x:v>
+      </x:c>
+      <x:c r="B8" s="95" t="str">
+        <x:v>Design baseline</x:v>
+      </x:c>
+      <x:c r="C8" s="95" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="D8" s="95" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E8" s="95" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="F8" s="95" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G8" s="95" t="str">
+        <x:v>Design constraints accepted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="50" customHeight="1">
+      <x:c r="A9" s="99" t="str">
+        <x:v>G01</x:v>
+      </x:c>
+      <x:c r="B9" s="95" t="str">
+        <x:v>Acceptance &amp; contracts</x:v>
+      </x:c>
+      <x:c r="C9" s="95" t="str">
+        <x:v>T02, T03, T04</x:v>
+      </x:c>
+      <x:c r="D9" s="95" t="str">
+        <x:v>After T02 approval, T03 and T04 are independent</x:v>
+      </x:c>
+      <x:c r="E9" s="95" t="str">
+        <x:v>T02 -&gt; review -&gt; T03 / T04</x:v>
+      </x:c>
+      <x:c r="F9" s="95" t="str">
+        <x:v>T01 approved</x:v>
+      </x:c>
+      <x:c r="G9" s="95" t="str">
+        <x:v>T02-T04 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="50" customHeight="1">
+      <x:c r="A10" s="99" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="B10" s="95" t="str">
+        <x:v>RabbitMQ transport core</x:v>
+      </x:c>
+      <x:c r="C10" s="95" t="str">
+        <x:v>T05, T06, T07, T08, T09</x:v>
+      </x:c>
+      <x:c r="D10" s="95" t="str">
+        <x:v>After T06 approval, T07 and T08 are independent</x:v>
+      </x:c>
+      <x:c r="E10" s="95" t="str">
+        <x:v>T05 -&gt; T06 -&gt; T07 / T08 -&gt; T09</x:v>
+      </x:c>
+      <x:c r="F10" s="95" t="str">
+        <x:v>T04 approved</x:v>
+      </x:c>
+      <x:c r="G10" s="95" t="str">
+        <x:v>T05-T09 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="50" customHeight="1">
+      <x:c r="A11" s="99" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="B11" s="95" t="str">
+        <x:v>Durable and worker foundations</x:v>
+      </x:c>
+      <x:c r="C11" s="95" t="str">
+        <x:v>T10, T14, T15, T16, T17</x:v>
+      </x:c>
+      <x:c r="D11" s="95" t="str">
+        <x:v>T10 and T14 can run independently; after T14, T15-T17 are independent</x:v>
+      </x:c>
+      <x:c r="E11" s="95" t="str">
+        <x:v>T10 / T14 -&gt; T15 / T16 / T17</x:v>
+      </x:c>
+      <x:c r="F11" s="95" t="str">
+        <x:v>Relevant G01-G02 dependencies approved</x:v>
+      </x:c>
+      <x:c r="G11" s="95" t="str">
+        <x:v>T10 and T14-T17 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="50" customHeight="1">
+      <x:c r="A12" s="99" t="str">
+        <x:v>G04</x:v>
+      </x:c>
+      <x:c r="B12" s="95" t="str">
+        <x:v>Relay &amp; audio happy path</x:v>
+      </x:c>
+      <x:c r="C12" s="95" t="str">
+        <x:v>T11, T18</x:v>
+      </x:c>
+      <x:c r="D12" s="95" t="str">
+        <x:v>T11 and T18 are independent once their own prerequisites pass</x:v>
+      </x:c>
+      <x:c r="E12" s="95" t="str">
+        <x:v>T11 / T18</x:v>
+      </x:c>
+      <x:c r="F12" s="95" t="str">
+        <x:v>G02-G03 prerequisites approved</x:v>
+      </x:c>
+      <x:c r="G12" s="95" t="str">
+        <x:v>T11 and T18 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
+      <x:c r="A13" s="99" t="str">
+        <x:v>G05</x:v>
+      </x:c>
+      <x:c r="B13" s="95" t="str">
+        <x:v>Producer facts &amp; idempotency</x:v>
+      </x:c>
+      <x:c r="C13" s="95" t="str">
+        <x:v>T12, T13, T19</x:v>
+      </x:c>
+      <x:c r="D13" s="95" t="str">
+        <x:v>All three tasks are independent</x:v>
+      </x:c>
+      <x:c r="E13" s="95" t="str">
+        <x:v>T12 / T13 / T19</x:v>
+      </x:c>
+      <x:c r="F13" s="95" t="str">
+        <x:v>T11 and T18 approved as applicable</x:v>
+      </x:c>
+      <x:c r="G13" s="95" t="str">
+        <x:v>T12, T13 and T19 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="50" customHeight="1">
+      <x:c r="A14" s="99" t="str">
+        <x:v>G06</x:v>
+      </x:c>
+      <x:c r="B14" s="95" t="str">
+        <x:v>Reliability &amp; downstream entry</x:v>
+      </x:c>
+      <x:c r="C14" s="95" t="str">
+        <x:v>T20, T22, T26</x:v>
+      </x:c>
+      <x:c r="D14" s="95" t="str">
+        <x:v>All three tasks are independent</x:v>
+      </x:c>
+      <x:c r="E14" s="95" t="str">
+        <x:v>T20 / T22 / T26</x:v>
+      </x:c>
+      <x:c r="F14" s="95" t="str">
+        <x:v>G05 task dependencies approved</x:v>
+      </x:c>
+      <x:c r="G14" s="95" t="str">
+        <x:v>T20, T22 and T26 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="50" customHeight="1">
+      <x:c r="A15" s="99" t="str">
+        <x:v>G07</x:v>
+      </x:c>
+      <x:c r="B15" s="95" t="str">
+        <x:v>State, AI contract &amp; identities</x:v>
+      </x:c>
+      <x:c r="C15" s="95" t="str">
+        <x:v>T21, T23, T27</x:v>
+      </x:c>
+      <x:c r="D15" s="95" t="str">
+        <x:v>All three tasks are independent</x:v>
+      </x:c>
+      <x:c r="E15" s="95" t="str">
+        <x:v>T21 / T23 / T27</x:v>
+      </x:c>
+      <x:c r="F15" s="95" t="str">
+        <x:v>G06 task dependencies approved</x:v>
+      </x:c>
+      <x:c r="G15" s="95" t="str">
+        <x:v>T21, T23 and T27 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="50" customHeight="1">
+      <x:c r="A16" s="99" t="str">
+        <x:v>G08</x:v>
+      </x:c>
+      <x:c r="B16" s="95" t="str">
+        <x:v>Corrections &amp; PHI safety</x:v>
+      </x:c>
+      <x:c r="C16" s="95" t="str">
+        <x:v>T24, T28</x:v>
+      </x:c>
+      <x:c r="D16" s="95" t="str">
+        <x:v>Both tasks are independent</x:v>
+      </x:c>
+      <x:c r="E16" s="95" t="str">
+        <x:v>T24 / T28</x:v>
+      </x:c>
+      <x:c r="F16" s="95" t="str">
+        <x:v>T23 and T27 approved</x:v>
+      </x:c>
+      <x:c r="G16" s="95" t="str">
+        <x:v>T24 and T28 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="50" customHeight="1">
+      <x:c r="A17" s="99" t="str">
+        <x:v>G09</x:v>
+      </x:c>
+      <x:c r="B17" s="95" t="str">
+        <x:v>Deletion &amp; operations</x:v>
+      </x:c>
+      <x:c r="C17" s="95" t="str">
+        <x:v>T25, T29, T30</x:v>
+      </x:c>
+      <x:c r="D17" s="95" t="str">
+        <x:v>After T25 approval, T29 and T30 are independent</x:v>
+      </x:c>
+      <x:c r="E17" s="95" t="str">
+        <x:v>T25 -&gt; T29 / T30</x:v>
+      </x:c>
+      <x:c r="F17" s="95" t="str">
+        <x:v>T21, T24 and T28 approved</x:v>
+      </x:c>
+      <x:c r="G17" s="95" t="str">
+        <x:v>T25, T29 and T30 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="50" customHeight="1">
+      <x:c r="A18" s="99" t="str">
+        <x:v>G10</x:v>
+      </x:c>
+      <x:c r="B18" s="95" t="str">
+        <x:v>Containers, scaling &amp; recovery</x:v>
+      </x:c>
+      <x:c r="C18" s="95" t="str">
+        <x:v>T31, T32, T33</x:v>
+      </x:c>
+      <x:c r="D18" s="95" t="str">
+        <x:v>After T31 approval, T32 and T33 are independent</x:v>
+      </x:c>
+      <x:c r="E18" s="95" t="str">
+        <x:v>T31 -&gt; T32 / T33</x:v>
+      </x:c>
+      <x:c r="F18" s="95" t="str">
+        <x:v>T29 and T30 approved</x:v>
+      </x:c>
+      <x:c r="G18" s="95" t="str">
+        <x:v>T31-T33 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="50" customHeight="1">
+      <x:c r="A19" s="99" t="str">
+        <x:v>G11</x:v>
+      </x:c>
+      <x:c r="B19" s="95" t="str">
+        <x:v>End-to-end verification</x:v>
+      </x:c>
+      <x:c r="C19" s="95" t="str">
+        <x:v>T34, T35</x:v>
+      </x:c>
+      <x:c r="D19" s="95" t="str">
+        <x:v>Sequential because T35 uses the completed failure matrix</x:v>
+      </x:c>
+      <x:c r="E19" s="95" t="str">
+        <x:v>T34 -&gt; T35</x:v>
+      </x:c>
+      <x:c r="F19" s="95" t="str">
+        <x:v>T31-T33 approved</x:v>
+      </x:c>
+      <x:c r="G19" s="95" t="str">
+        <x:v>T34 and T35 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="50" customHeight="1">
+      <x:c r="A20" s="99" t="str">
+        <x:v>G12</x:v>
+      </x:c>
+      <x:c r="B20" s="95" t="str">
+        <x:v>Legacy removal &amp; release</x:v>
+      </x:c>
+      <x:c r="C20" s="95" t="str">
+        <x:v>T36, T37</x:v>
+      </x:c>
+      <x:c r="D20" s="95" t="str">
+        <x:v>Sequential release gate</x:v>
+      </x:c>
+      <x:c r="E20" s="95" t="str">
+        <x:v>T36 -&gt; T37</x:v>
+      </x:c>
+      <x:c r="F20" s="95" t="str">
+        <x:v>T34 and T35 approved</x:v>
+      </x:c>
+      <x:c r="G20" s="95" t="str">
+        <x:v>T36 and T37 approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="A22" s="100" t="str">
+        <x:v>Per-task review queue</x:v>
+      </x:c>
+      <x:c r="B22" s="100"/>
+      <x:c r="C22" s="100"/>
+      <x:c r="D22" s="100"/>
+      <x:c r="E22" s="100"/>
+      <x:c r="F22" s="100"/>
+      <x:c r="G22" s="100"/>
+      <x:c r="H22" s="100"/>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="79" t="str">
+        <x:v>Task ID</x:v>
+      </x:c>
+      <x:c r="B23" s="79" t="str">
+        <x:v>Group</x:v>
+      </x:c>
+      <x:c r="C23" s="79" t="str">
+        <x:v>Phase</x:v>
+      </x:c>
+      <x:c r="D23" s="79" t="str">
+        <x:v>Title</x:v>
+      </x:c>
+      <x:c r="E23" s="79" t="str">
+        <x:v>Depends On</x:v>
+      </x:c>
+      <x:c r="F23" s="79" t="str">
+        <x:v>Work Status</x:v>
+      </x:c>
+      <x:c r="G23" s="79" t="str">
+        <x:v>Code Review</x:v>
+      </x:c>
+      <x:c r="H23" s="79" t="str">
+        <x:v>Review commit / notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="99" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="B24" s="95" t="str">
+        <x:v>G00</x:v>
+      </x:c>
+      <x:c r="C24" s="95" t="str">
+        <x:v>0 - Foundations</x:v>
+      </x:c>
+      <x:c r="D24" s="95" t="str">
+        <x:v>Design documentation</x:v>
+      </x:c>
+      <x:c r="E24" s="95"/>
+      <x:c r="F24" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A24,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G24" s="101" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="H24" s="101" t="str"/>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="99" t="str">
+        <x:v>T02</x:v>
+      </x:c>
+      <x:c r="B25" s="95" t="str">
+        <x:v>G01</x:v>
+      </x:c>
+      <x:c r="C25" s="95" t="str">
+        <x:v>0 - Foundations</x:v>
+      </x:c>
+      <x:c r="D25" s="95" t="str">
+        <x:v>Root Compose acceptance seam</x:v>
+      </x:c>
+      <x:c r="E25" s="95" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="F25" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A25,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G25" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H25" s="101" t="str"/>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="99" t="str">
+        <x:v>T03</x:v>
+      </x:c>
+      <x:c r="B26" s="95" t="str">
+        <x:v>G01</x:v>
+      </x:c>
+      <x:c r="C26" s="95" t="str">
+        <x:v>0 - Foundations</x:v>
+      </x:c>
+      <x:c r="D26" s="95" t="str">
+        <x:v>Persistence schema &amp; migration ownership</x:v>
+      </x:c>
+      <x:c r="E26" s="95" t="str">
+        <x:v>T02</x:v>
+      </x:c>
+      <x:c r="F26" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A26,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G26" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H26" s="101" t="str"/>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="99" t="str">
+        <x:v>T04</x:v>
+      </x:c>
+      <x:c r="B27" s="95" t="str">
+        <x:v>G01</x:v>
+      </x:c>
+      <x:c r="C27" s="95" t="str">
+        <x:v>1 - Event Bus Core</x:v>
+      </x:c>
+      <x:c r="D27" s="95" t="str">
+        <x:v>Integration-event envelope &amp; stable names</x:v>
+      </x:c>
+      <x:c r="E27" s="95" t="str">
+        <x:v>T02</x:v>
+      </x:c>
+      <x:c r="F27" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A27,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G27" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H27" s="101" t="str"/>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="99" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="B28" s="95" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="C28" s="95" t="str">
+        <x:v>1 - Event Bus Core</x:v>
+      </x:c>
+      <x:c r="D28" s="95" t="str">
+        <x:v>Typed handlers &amp; subscription registry</x:v>
+      </x:c>
+      <x:c r="E28" s="95" t="str">
+        <x:v>T04</x:v>
+      </x:c>
+      <x:c r="F28" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A28,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G28" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H28" s="101" t="str"/>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="99" t="str">
+        <x:v>T06</x:v>
+      </x:c>
+      <x:c r="B29" s="95" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="C29" s="95" t="str">
+        <x:v>1 - Event Bus Core</x:v>
+      </x:c>
+      <x:c r="D29" s="95" t="str">
+        <x:v>RabbitMQ connection &amp; hosted consumer</x:v>
+      </x:c>
+      <x:c r="E29" s="95" t="str">
+        <x:v>T04, T05</x:v>
+      </x:c>
+      <x:c r="F29" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A29,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G29" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H29" s="101" t="str"/>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="99" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="B30" s="95" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="C30" s="95" t="str">
+        <x:v>1 - Event Bus Core</x:v>
+      </x:c>
+      <x:c r="D30" s="95" t="str">
+        <x:v>Exchange and subscriber-owned topology</x:v>
+      </x:c>
+      <x:c r="E30" s="95" t="str">
+        <x:v>T06</x:v>
+      </x:c>
+      <x:c r="F30" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A30,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G30" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H30" s="101" t="str"/>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="99" t="str">
+        <x:v>T08</x:v>
+      </x:c>
+      <x:c r="B31" s="95" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="C31" s="95" t="str">
+        <x:v>1 - Event Bus Core</x:v>
+      </x:c>
+      <x:c r="D31" s="95" t="str">
+        <x:v>Confirmed publisher &amp; trace propagation</x:v>
+      </x:c>
+      <x:c r="E31" s="95" t="str">
+        <x:v>T04, T06</x:v>
+      </x:c>
+      <x:c r="F31" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A31,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G31" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H31" s="101" t="str"/>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="99" t="str">
+        <x:v>T09</x:v>
+      </x:c>
+      <x:c r="B32" s="95" t="str">
+        <x:v>G02</x:v>
+      </x:c>
+      <x:c r="C32" s="95" t="str">
+        <x:v>1 - Event Bus Core</x:v>
+      </x:c>
+      <x:c r="D32" s="95" t="str">
+        <x:v>Wire-contract and topology tests</x:v>
+      </x:c>
+      <x:c r="E32" s="95" t="str">
+        <x:v>T04, T07, T08</x:v>
+      </x:c>
+      <x:c r="F32" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A32,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G32" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H32" s="101" t="str"/>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="99" t="str">
+        <x:v>T10</x:v>
+      </x:c>
+      <x:c r="B33" s="95" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="C33" s="95" t="str">
+        <x:v>2 - Durable Publication</x:v>
+      </x:c>
+      <x:c r="D33" s="95" t="str">
+        <x:v>Transactional outbox write path</x:v>
+      </x:c>
+      <x:c r="E33" s="95" t="str">
+        <x:v>T03, T04</x:v>
+      </x:c>
+      <x:c r="F33" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A33,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G33" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H33" s="101" t="str"/>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="99" t="str">
+        <x:v>T11</x:v>
+      </x:c>
+      <x:c r="B34" s="95" t="str">
+        <x:v>G04</x:v>
+      </x:c>
+      <x:c r="C34" s="95" t="str">
+        <x:v>2 - Durable Publication</x:v>
+      </x:c>
+      <x:c r="D34" s="95" t="str">
+        <x:v>Continuous outbox relay</x:v>
+      </x:c>
+      <x:c r="E34" s="95" t="str">
+        <x:v>T08, T10</x:v>
+      </x:c>
+      <x:c r="F34" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A34,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G34" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H34" s="101" t="str"/>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="99" t="str">
+        <x:v>T12</x:v>
+      </x:c>
+      <x:c r="B35" s="95" t="str">
+        <x:v>G05</x:v>
+      </x:c>
+      <x:c r="C35" s="95" t="str">
+        <x:v>2 - Durable Publication</x:v>
+      </x:c>
+      <x:c r="D35" s="95" t="str">
+        <x:v>Audio and document upload events</x:v>
+      </x:c>
+      <x:c r="E35" s="95" t="str">
+        <x:v>T09, T10, T11</x:v>
+      </x:c>
+      <x:c r="F35" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A35,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G35" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H35" s="101" t="str"/>
+    </x:row>
+    <x:row r="36" ht="34" customHeight="1">
+      <x:c r="A36" s="99" t="str">
+        <x:v>T13</x:v>
+      </x:c>
+      <x:c r="B36" s="95" t="str">
+        <x:v>G05</x:v>
+      </x:c>
+      <x:c r="C36" s="95" t="str">
+        <x:v>2 - Durable Publication</x:v>
+      </x:c>
+      <x:c r="D36" s="95" t="str">
+        <x:v>Transcript revision and deletion events</x:v>
+      </x:c>
+      <x:c r="E36" s="95" t="str">
+        <x:v>T09, T10, T11</x:v>
+      </x:c>
+      <x:c r="F36" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A36,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G36" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H36" s="101" t="str"/>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="99" t="str">
+        <x:v>T14</x:v>
+      </x:c>
+      <x:c r="B37" s="95" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="C37" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D37" s="95" t="str">
+        <x:v>Standard Transcription Worker host</x:v>
+      </x:c>
+      <x:c r="E37" s="95" t="str">
+        <x:v>T06, T07</x:v>
+      </x:c>
+      <x:c r="F37" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A37,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G37" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H37" s="101" t="str"/>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="99" t="str">
+        <x:v>T15</x:v>
+      </x:c>
+      <x:c r="B38" s="95" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="C38" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D38" s="95" t="str">
+        <x:v>Restricted shared-database unit of work</x:v>
+      </x:c>
+      <x:c r="E38" s="95" t="str">
+        <x:v>T03, T14</x:v>
+      </x:c>
+      <x:c r="F38" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A38,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G38" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H38" s="101" t="str"/>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="99" t="str">
+        <x:v>T16</x:v>
+      </x:c>
+      <x:c r="B39" s="95" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="C39" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D39" s="95" t="str">
+        <x:v>Private Blob retrieval adapter</x:v>
+      </x:c>
+      <x:c r="E39" s="95" t="str">
+        <x:v>T14</x:v>
+      </x:c>
+      <x:c r="F39" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A39,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G39" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H39" s="101" t="str"/>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="99" t="str">
+        <x:v>T17</x:v>
+      </x:c>
+      <x:c r="B40" s="95" t="str">
+        <x:v>G03</x:v>
+      </x:c>
+      <x:c r="C40" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D40" s="95" t="str">
+        <x:v>Azure Speech adapter &amp; safe failures</x:v>
+      </x:c>
+      <x:c r="E40" s="95" t="str">
+        <x:v>T14</x:v>
+      </x:c>
+      <x:c r="F40" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A40,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G40" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H40" s="101" t="str"/>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="99" t="str">
+        <x:v>T18</x:v>
+      </x:c>
+      <x:c r="B41" s="95" t="str">
+        <x:v>G04</x:v>
+      </x:c>
+      <x:c r="C41" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D41" s="95" t="str">
+        <x:v>Audio Uploaded happy path</x:v>
+      </x:c>
+      <x:c r="E41" s="95" t="str">
+        <x:v>T09, T15, T16, T17</x:v>
+      </x:c>
+      <x:c r="F41" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A41,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G41" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H41" s="101" t="str"/>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="99" t="str">
+        <x:v>T19</x:v>
+      </x:c>
+      <x:c r="B42" s="95" t="str">
+        <x:v>G05</x:v>
+      </x:c>
+      <x:c r="C42" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D42" s="95" t="str">
+        <x:v>Inbox idempotency &amp; crash redelivery</x:v>
+      </x:c>
+      <x:c r="E42" s="95" t="str">
+        <x:v>T18</x:v>
+      </x:c>
+      <x:c r="F42" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A42,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G42" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H42" s="101" t="str"/>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="99" t="str">
+        <x:v>T20</x:v>
+      </x:c>
+      <x:c r="B43" s="95" t="str">
+        <x:v>G06</x:v>
+      </x:c>
+      <x:c r="C43" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D43" s="95" t="str">
+        <x:v>Retry, dead-letter &amp; failure classification</x:v>
+      </x:c>
+      <x:c r="E43" s="95" t="str">
+        <x:v>T18, T19</x:v>
+      </x:c>
+      <x:c r="F43" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A43,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G43" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H43" s="101" t="str"/>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="99" t="str">
+        <x:v>T21</x:v>
+      </x:c>
+      <x:c r="B44" s="95" t="str">
+        <x:v>G07</x:v>
+      </x:c>
+      <x:c r="C44" s="95" t="str">
+        <x:v>3 - Transcription Worker</x:v>
+      </x:c>
+      <x:c r="D44" s="95" t="str">
+        <x:v>State gates, concurrency &amp; shutdown</x:v>
+      </x:c>
+      <x:c r="E44" s="95" t="str">
+        <x:v>T18, T19, T20</x:v>
+      </x:c>
+      <x:c r="F44" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A44,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G44" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H44" s="101" t="str"/>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="99" t="str">
+        <x:v>T22</x:v>
+      </x:c>
+      <x:c r="B45" s="95" t="str">
+        <x:v>G06</x:v>
+      </x:c>
+      <x:c r="C45" s="95" t="str">
+        <x:v>4 - Downstream &amp; Deletion</x:v>
+      </x:c>
+      <x:c r="D45" s="95" t="str">
+        <x:v>Backend Transcript Ready subscriber</x:v>
+      </x:c>
+      <x:c r="E45" s="95" t="str">
+        <x:v>T09, T13, T18</x:v>
+      </x:c>
+      <x:c r="F45" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A45,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G45" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H45" s="101" t="str"/>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="99" t="str">
+        <x:v>T23</x:v>
+      </x:c>
+      <x:c r="B46" s="95" t="str">
+        <x:v>G07</x:v>
+      </x:c>
+      <x:c r="C46" s="95" t="str">
+        <x:v>4 - Downstream &amp; Deletion</x:v>
+      </x:c>
+      <x:c r="D46" s="95" t="str">
+        <x:v>Current Clinical Knowledge contract alignment</x:v>
+      </x:c>
+      <x:c r="E46" s="95" t="str">
+        <x:v>T22</x:v>
+      </x:c>
+      <x:c r="F46" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A46,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G46" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H46" s="101" t="str"/>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="99" t="str">
+        <x:v>T24</x:v>
+      </x:c>
+      <x:c r="B47" s="95" t="str">
+        <x:v>G08</x:v>
+      </x:c>
+      <x:c r="C47" s="95" t="str">
+        <x:v>4 - Downstream &amp; Deletion</x:v>
+      </x:c>
+      <x:c r="D47" s="95" t="str">
+        <x:v>Idempotent Ingestion handoff &amp; correction</x:v>
+      </x:c>
+      <x:c r="E47" s="95" t="str">
+        <x:v>T22, T23</x:v>
+      </x:c>
+      <x:c r="F47" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A47,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G47" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H47" s="101" t="str"/>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="99" t="str">
+        <x:v>T25</x:v>
+      </x:c>
+      <x:c r="B48" s="95" t="str">
+        <x:v>G09</x:v>
+      </x:c>
+      <x:c r="C48" s="95" t="str">
+        <x:v>4 - Downstream &amp; Deletion</x:v>
+      </x:c>
+      <x:c r="D48" s="95" t="str">
+        <x:v>Event-driven deletion cleanup</x:v>
+      </x:c>
+      <x:c r="E48" s="95" t="str">
+        <x:v>T13, T21, T24</x:v>
+      </x:c>
+      <x:c r="F48" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A48,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G48" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H48" s="101" t="str"/>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="99" t="str">
+        <x:v>T26</x:v>
+      </x:c>
+      <x:c r="B49" s="95" t="str">
+        <x:v>G06</x:v>
+      </x:c>
+      <x:c r="C49" s="95" t="str">
+        <x:v>4 - Downstream &amp; Deletion</x:v>
+      </x:c>
+      <x:c r="D49" s="95" t="str">
+        <x:v>Document pending behavior</x:v>
+      </x:c>
+      <x:c r="E49" s="95" t="str">
+        <x:v>T12, T14, T18</x:v>
+      </x:c>
+      <x:c r="F49" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A49,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G49" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H49" s="101" t="str"/>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="99" t="str">
+        <x:v>T27</x:v>
+      </x:c>
+      <x:c r="B50" s="95" t="str">
+        <x:v>G07</x:v>
+      </x:c>
+      <x:c r="C50" s="95" t="str">
+        <x:v>5 - Security &amp; Observability</x:v>
+      </x:c>
+      <x:c r="D50" s="95" t="str">
+        <x:v>Service identities, TLS &amp; secrets</x:v>
+      </x:c>
+      <x:c r="E50" s="95" t="str">
+        <x:v>T07, T14</x:v>
+      </x:c>
+      <x:c r="F50" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A50,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G50" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H50" s="101" t="str"/>
+    </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="99" t="str">
+        <x:v>T28</x:v>
+      </x:c>
+      <x:c r="B51" s="95" t="str">
+        <x:v>G08</x:v>
+      </x:c>
+      <x:c r="C51" s="95" t="str">
+        <x:v>5 - Security &amp; Observability</x:v>
+      </x:c>
+      <x:c r="D51" s="95" t="str">
+        <x:v>PHI-safe telemetry &amp; canary tests</x:v>
+      </x:c>
+      <x:c r="E51" s="95" t="str">
+        <x:v>T17, T18, T22, T27</x:v>
+      </x:c>
+      <x:c r="F51" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A51,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G51" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H51" s="101" t="str"/>
+    </x:row>
+    <x:row r="52" ht="34" customHeight="1">
+      <x:c r="A52" s="99" t="str">
+        <x:v>T29</x:v>
+      </x:c>
+      <x:c r="B52" s="95" t="str">
+        <x:v>G09</x:v>
+      </x:c>
+      <x:c r="C52" s="95" t="str">
+        <x:v>5 - Security &amp; Observability</x:v>
+      </x:c>
+      <x:c r="D52" s="95" t="str">
+        <x:v>Health, metrics, dashboards &amp; alerts</x:v>
+      </x:c>
+      <x:c r="E52" s="95" t="str">
+        <x:v>T11, T20, T22, T25, T28</x:v>
+      </x:c>
+      <x:c r="F52" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A52,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G52" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H52" s="101" t="str"/>
+    </x:row>
+    <x:row r="53" ht="34" customHeight="1">
+      <x:c r="A53" s="99" t="str">
+        <x:v>T30</x:v>
+      </x:c>
+      <x:c r="B53" s="95" t="str">
+        <x:v>G09</x:v>
+      </x:c>
+      <x:c r="C53" s="95" t="str">
+        <x:v>5 - Security &amp; Observability</x:v>
+      </x:c>
+      <x:c r="D53" s="95" t="str">
+        <x:v>Retention, audit &amp; replay authorization</x:v>
+      </x:c>
+      <x:c r="E53" s="95" t="str">
+        <x:v>T20, T25, T27, T28</x:v>
+      </x:c>
+      <x:c r="F53" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A53,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G53" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H53" s="101" t="str"/>
+    </x:row>
+    <x:row r="54" ht="34" customHeight="1">
+      <x:c r="A54" s="99" t="str">
+        <x:v>T31</x:v>
+      </x:c>
+      <x:c r="B54" s="95" t="str">
+        <x:v>G10</x:v>
+      </x:c>
+      <x:c r="C54" s="95" t="str">
+        <x:v>6 - Containers &amp; Operations</x:v>
+      </x:c>
+      <x:c r="D54" s="95" t="str">
+        <x:v>Dockerfiles &amp; root Compose stack</x:v>
+      </x:c>
+      <x:c r="E54" s="95" t="str">
+        <x:v>T14, T22, T27</x:v>
+      </x:c>
+      <x:c r="F54" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A54,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G54" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H54" s="101" t="str"/>
+    </x:row>
+    <x:row r="55" ht="34" customHeight="1">
+      <x:c r="A55" s="99" t="str">
+        <x:v>T32</x:v>
+      </x:c>
+      <x:c r="B55" s="95" t="str">
+        <x:v>G10</x:v>
+      </x:c>
+      <x:c r="C55" s="95" t="str">
+        <x:v>6 - Containers &amp; Operations</x:v>
+      </x:c>
+      <x:c r="D55" s="95" t="str">
+        <x:v>Scaling and deployment behavior</x:v>
+      </x:c>
+      <x:c r="E55" s="95" t="str">
+        <x:v>T21, T29, T31</x:v>
+      </x:c>
+      <x:c r="F55" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A55,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G55" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H55" s="101" t="str"/>
+    </x:row>
+    <x:row r="56" ht="34" customHeight="1">
+      <x:c r="A56" s="99" t="str">
+        <x:v>T33</x:v>
+      </x:c>
+      <x:c r="B56" s="95" t="str">
+        <x:v>G10</x:v>
+      </x:c>
+      <x:c r="C56" s="95" t="str">
+        <x:v>6 - Containers &amp; Operations</x:v>
+      </x:c>
+      <x:c r="D56" s="95" t="str">
+        <x:v>DLQ replay &amp; recovery tooling</x:v>
+      </x:c>
+      <x:c r="E56" s="95" t="str">
+        <x:v>T20, T29, T30, T31</x:v>
+      </x:c>
+      <x:c r="F56" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A56,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G56" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H56" s="101" t="str"/>
+    </x:row>
+    <x:row r="57" ht="34" customHeight="1">
+      <x:c r="A57" s="99" t="str">
+        <x:v>T34</x:v>
+      </x:c>
+      <x:c r="B57" s="95" t="str">
+        <x:v>G11</x:v>
+      </x:c>
+      <x:c r="C57" s="95" t="str">
+        <x:v>7 - Verification &amp; Removal</x:v>
+      </x:c>
+      <x:c r="D57" s="95" t="str">
+        <x:v>End-to-end failure matrix</x:v>
+      </x:c>
+      <x:c r="E57" s="95" t="str">
+        <x:v>T31, T32, T33</x:v>
+      </x:c>
+      <x:c r="F57" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A57,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G57" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H57" s="101" t="str"/>
+    </x:row>
+    <x:row r="58" ht="34" customHeight="1">
+      <x:c r="A58" s="99" t="str">
+        <x:v>T35</x:v>
+      </x:c>
+      <x:c r="B58" s="95" t="str">
+        <x:v>G11</x:v>
+      </x:c>
+      <x:c r="C58" s="95" t="str">
+        <x:v>7 - Verification &amp; Removal</x:v>
+      </x:c>
+      <x:c r="D58" s="95" t="str">
+        <x:v>Architecture and privacy enforcement</x:v>
+      </x:c>
+      <x:c r="E58" s="95" t="str">
+        <x:v>T28, T34</x:v>
+      </x:c>
+      <x:c r="F58" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A58,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G58" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H58" s="101" t="str"/>
+    </x:row>
+    <x:row r="59" ht="34" customHeight="1">
+      <x:c r="A59" s="99" t="str">
+        <x:v>T36</x:v>
+      </x:c>
+      <x:c r="B59" s="95" t="str">
+        <x:v>G12</x:v>
+      </x:c>
+      <x:c r="C59" s="95" t="str">
+        <x:v>7 - Verification &amp; Removal</x:v>
+      </x:c>
+      <x:c r="D59" s="95" t="str">
+        <x:v>Remove Function and legacy messaging</x:v>
+      </x:c>
+      <x:c r="E59" s="95" t="str">
+        <x:v>T34, T35</x:v>
+      </x:c>
+      <x:c r="F59" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A59,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G59" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H59" s="101" t="str"/>
+    </x:row>
+    <x:row r="60" ht="34" customHeight="1">
+      <x:c r="A60" s="99" t="str">
+        <x:v>T37</x:v>
+      </x:c>
+      <x:c r="B60" s="95" t="str">
+        <x:v>G12</x:v>
+      </x:c>
+      <x:c r="C60" s="95" t="str">
+        <x:v>7 - Verification &amp; Removal</x:v>
+      </x:c>
+      <x:c r="D60" s="95" t="str">
+        <x:v>Clean-environment release gate</x:v>
+      </x:c>
+      <x:c r="E60" s="95" t="str">
+        <x:v>T36</x:v>
+      </x:c>
+      <x:c r="F60" s="95" t="str">
+        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A60,'Tasks'!$A$2:$A$38,0))</x:f>
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="G60" s="101" t="str">
+        <x:v>Not Submitted</x:v>
+      </x:c>
+      <x:c r="H60" s="101" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H3"/>
+    <x:mergeCell ref="A22:H22"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="G24:G60">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Approved"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="In Review"/>
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Changes Requested"/>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Not Submitted"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G24:G60">
+      <x:formula1>"Not Submitted,In Review,Changes Requested,Approved"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d0b2de16fac45d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57531d8bf1254f7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T04 add stable integration event contracts
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1522,7 +1522,7 @@
       </c>
       <c r="G5" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="92" min="1" max="1"/>
@@ -3633,16 +3633,21 @@
           <t>T02</t>
         </is>
       </c>
-      <c r="F27" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A27,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F27" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G27" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H27" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H27" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="34" customHeight="1" s="92">
       <c r="A28" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T05 add typed event handler dispatch
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1559,7 +1559,7 @@
       </c>
       <c r="G6" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3675,16 +3675,21 @@
           <t>T04</t>
         </is>
       </c>
-      <c r="F28" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A28,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F28" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G28" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H28" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H28" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="34" customHeight="1" s="92">
       <c r="A29" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T06 add RabbitMQ hosted consumer
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1596,7 +1596,7 @@
       </c>
       <c r="G7" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3717,16 +3717,21 @@
           <t>T04, T05</t>
         </is>
       </c>
-      <c r="F29" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A29,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F29" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G29" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H29" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H29" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="34" customHeight="1" s="92">
       <c r="A30" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T07 add RabbitMQ subscriber topology
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G8" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3759,16 +3759,21 @@
           <t>T06</t>
         </is>
       </c>
-      <c r="F30" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A30,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F30" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G30" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H30" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H30" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="34" customHeight="1" s="92">
       <c r="A31" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T08 add confirmed RabbitMQ publisher
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1670,7 +1670,7 @@
       </c>
       <c r="G9" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3801,16 +3801,21 @@
           <t>T04, T06</t>
         </is>
       </c>
-      <c r="F31" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A31,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F31" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G31" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H31" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H31" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="34" customHeight="1" s="92">
       <c r="A32" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T09 add event bus wire contract tests
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G10" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3843,16 +3843,21 @@
           <t>T04, T07, T08</t>
         </is>
       </c>
-      <c r="F32" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A32,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F32" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G32" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H32" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H32" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available. Live broker execution requires Docker availability.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="34" customHeight="1" s="92">
       <c r="A33" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T10 stage upload events in outbox
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1744,7 +1744,7 @@
       </c>
       <c r="G11" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3885,16 +3885,21 @@
           <t>T03, T04</t>
         </is>
       </c>
-      <c r="F33" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A33,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F33" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G33" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H33" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H33" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="34" customHeight="1" s="92">
       <c r="A34" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T11 add continuous outbox relay
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1781,7 +1781,7 @@
       </c>
       <c r="G12" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3927,16 +3927,21 @@
           <t>T08, T10</t>
         </is>
       </c>
-      <c r="F34" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A34,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F34" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G34" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H34" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H34" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available. Relay hosted service is config-gated.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="34" customHeight="1" s="92">
       <c r="A35" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T12 verify upload event payloads
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1818,7 +1818,7 @@
       </c>
       <c r="G13" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -3969,16 +3969,21 @@
           <t>T09, T10, T11</t>
         </is>
       </c>
-      <c r="F35" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A35,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F35" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G35" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H35" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H35" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="34" customHeight="1" s="92">
       <c r="A36" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T14 add standalone transcription worker host
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd0395b473ca44fa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R6d0535b94e7d4ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rae9166ea49514981"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R449131cefd584342"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbf1b6daab13a4d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R77ac058144c04bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rde9f73fa2e6340a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R4d7132ee16384511"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1205,16 +1205,13 @@
         </x:is>
       </x:c>
       <x:c r="C23" s="9" t="n">
-        <x:f>COUNTIF('Tasks'!$B$2:$B$999,B23)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:f>COUNTIFS('Tasks'!$B$2:$B$999,B23,'Tasks'!$G$2:$G$999,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:f>C23-D23</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1303,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1873,10 +1870,8 @@
           <x:t xml:space="preserve">T06, T07</x:t>
         </x:is>
       </x:c>
-      <x:c r="G15" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G15" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2817,7 +2812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e7d1db0f8394492"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5a3a12ef8bf4405"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4021,15 +4016,14 @@
         </x:is>
       </x:c>
       <x:c r="F37" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A37,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G37" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H37" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G37" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H37" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A38" s="99" t="inlineStr">
@@ -4901,8 +4895,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5297c0d565fe4bd2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3c9d4393d344b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf8c4b215f794eaa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc471efed34504988"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T15 add transcription completion unit of work
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rbf1b6daab13a4d62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R77ac058144c04bd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rde9f73fa2e6340a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R4d7132ee16384511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R86c82539fec64302"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R75dc0391fa66448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R729812786b004a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rbf2f7fc853004e06"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,10 +1208,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1300,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1905,10 +1905,8 @@
           <x:t xml:space="preserve">T03, T14</x:t>
         </x:is>
       </x:c>
-      <x:c r="G16" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G16" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2812,7 +2810,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5a3a12ef8bf4405"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bf36947076343f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4052,15 +4050,14 @@
         </x:is>
       </x:c>
       <x:c r="F38" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A38,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G38" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H38" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G38" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H38" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A39" s="99" t="inlineStr">
@@ -4895,8 +4892,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf8c4b215f794eaa"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc471efed34504988"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35cd8a497c0c4788"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5ff58deb0b54bb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T16 add private audio blob retrieval adapter
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R86c82539fec64302"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R75dc0391fa66448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R729812786b004a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rbf2f7fc853004e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra91a49b8248241c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R5dd8dbed8d0847ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rb2bc805c61db4fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R895b409296134285"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,10 +1208,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1300,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1940,10 +1940,8 @@
           <x:t xml:space="preserve">T14</x:t>
         </x:is>
       </x:c>
-      <x:c r="G17" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G17" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2810,7 +2808,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bf36947076343f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52a3e2f22a7148e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4086,15 +4084,14 @@
         </x:is>
       </x:c>
       <x:c r="F39" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A39,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G39" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H39" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G39" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H39" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A40" s="99" t="inlineStr">
@@ -4892,8 +4889,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35cd8a497c0c4788"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5ff58deb0b54bb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccf6a0e74bf457e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2a029d6d52f469f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T17 add Azure Speech transcription adapter
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra91a49b8248241c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R5dd8dbed8d0847ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rb2bc805c61db4fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R895b409296134285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd1c5a974faf942f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R954ada1f2f5449aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R1fbd3f8d9151458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rd906af17eee0469f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,10 +1208,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1300,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1975,10 +1975,8 @@
           <x:t xml:space="preserve">T14</x:t>
         </x:is>
       </x:c>
-      <x:c r="G18" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G18" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2808,7 +2806,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52a3e2f22a7148e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26f87b7d3ff5437a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4120,15 +4118,14 @@
         </x:is>
       </x:c>
       <x:c r="F40" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A40,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G40" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H40" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G40" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H40" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A41" s="99" t="inlineStr">
@@ -4889,8 +4886,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccf6a0e74bf457e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2a029d6d52f469f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d767cc1923c4989"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20444b02b0e84f64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T18 connect audio uploaded worker happy path
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd1c5a974faf942f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R954ada1f2f5449aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R1fbd3f8d9151458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rd906af17eee0469f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7c71435933e44e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rfcca492bebfc4e19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rebeffe0150d7408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rd163e6c3e76944b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,10 +1208,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1300,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2010,10 +2010,8 @@
           <x:t xml:space="preserve">T09, T15, T16, T17</x:t>
         </x:is>
       </x:c>
-      <x:c r="G19" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G19" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2806,7 +2804,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26f87b7d3ff5437a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f6ef4461d754308"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4154,15 +4152,14 @@
         </x:is>
       </x:c>
       <x:c r="F41" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A41,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G41" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H41" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G41" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H41" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A42" s="99" t="inlineStr">
@@ -4886,8 +4883,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d767cc1923c4989"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20444b02b0e84f64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc115579365e74059"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf10aac04fbd46b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T19 add transcription inbox idempotency claims
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7c71435933e44e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rfcca492bebfc4e19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rebeffe0150d7408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rd163e6c3e76944b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R14baef2040874b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Re6b797345c024788"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R35ffa748ef5a4926"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rbe96485f172d4c90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,10 +1208,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1300,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="n">
         <x:v>18</x:v>
-      </x:c>
-      <x:c r="E28" s="11" t="n">
-        <x:v>19</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2045,10 +2045,8 @@
           <x:t xml:space="preserve">T18</x:t>
         </x:is>
       </x:c>
-      <x:c r="G20" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G20" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2804,7 +2802,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f6ef4461d754308"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29ea163082047a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4188,15 +4186,14 @@
         </x:is>
       </x:c>
       <x:c r="F42" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A42,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G42" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H42" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G42" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H42" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A43" s="99" t="inlineStr">
@@ -4883,8 +4880,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc115579365e74059"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf10aac04fbd46b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f643a0d0b4b4bd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf77e25b8ab9042a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T20 classify transcription retry and failure outcomes
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R14baef2040874b7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Re6b797345c024788"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R35ffa748ef5a4926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rbe96485f172d4c90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R64fc5782ce674435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R391acaeab0ac46b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Ra403bcdf94114517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rc7ae1ae64e9345da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1208,10 +1208,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E23" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1300,10 +1300,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2080,10 +2080,8 @@
           <x:t xml:space="preserve">T18, T19</x:t>
         </x:is>
       </x:c>
-      <x:c r="G21" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G21" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="22" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2802,7 +2800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29ea163082047a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f3dce4a0b724c52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4222,15 +4220,14 @@
         </x:is>
       </x:c>
       <x:c r="F43" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A43,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G43" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H43" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G43" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H43" s="101" t="str">
+        <x:v>Committed for user review when available.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A44" s="99" t="inlineStr">
@@ -4880,8 +4877,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f643a0d0b4b4bd0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf77e25b8ab9042a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3421f9c44dad4c15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3640b55ad289459f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T22 add backend transcript ready subscriber
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1221,17 +1221,14 @@
           <t>4 - Downstream &amp; Deletion</t>
         </is>
       </c>
-      <c r="C24" s="9">
-        <f>COUNTIF('Tasks'!$B$2:$B$999,B24)</f>
-        <v/>
-      </c>
-      <c r="D24" s="9">
-        <f>COUNTIFS('Tasks'!$B$2:$B$999,B24,'Tasks'!$G$2:$G$999,"Completed")</f>
-        <v/>
-      </c>
-      <c r="E24" s="9">
-        <f>C24-D24</f>
-        <v/>
+      <c r="C24" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -1301,10 +1298,10 @@
         <v>37</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2176,7 +2173,7 @@
       </c>
       <c r="G23" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -4374,16 +4371,21 @@
           <t>T09, T13, T18</t>
         </is>
       </c>
-      <c r="F45" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A45,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F45" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G45" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H45" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H45" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="34" customHeight="1" s="92">
       <c r="A46" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T23 align transcript handoff with clinical knowledge ingestion
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Known Bugs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Implementation Plan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -1225,10 +1225,10 @@
         <v>5</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1298,10 +1298,10 @@
         <v>37</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="G24" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -4413,16 +4413,21 @@
           <t>T22</t>
         </is>
       </c>
-      <c r="F46" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A46,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F46" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G46" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H46" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H46" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="34" customHeight="1" s="92">
       <c r="A47" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T24 persist clinical knowledge ingestion handoff results
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1225,10 +1225,10 @@
         <v>5</v>
       </c>
       <c r="D24" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="9" t="n">
         <v>2</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1298,10 +1298,10 @@
         <v>37</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="G25" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -4455,16 +4455,21 @@
           <t>T22, T23</t>
         </is>
       </c>
-      <c r="F47" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A47,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F47" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G47" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H47" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H47" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="34" customHeight="1" s="92">
       <c r="A48" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T25 add event driven deletion cleanup
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -1225,10 +1225,10 @@
         <v>5</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1298,10 +1298,10 @@
         <v>37</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E28" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="G26" s="70" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -4497,16 +4497,21 @@
           <t>T13, T21, T24</t>
         </is>
       </c>
-      <c r="F48" s="95">
-        <f>INDEX('Tasks'!$G$2:$G$38,MATCH(A48,'Tasks'!$A$2:$A$38,0))</f>
-        <v/>
+      <c r="F48" s="95" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="G48" s="101" t="inlineStr">
         <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="H48" s="101" t="str"/>
+          <t>Review Deferred</t>
+        </is>
+      </c>
+      <c r="H48" s="101" t="inlineStr">
+        <is>
+          <t>Committed for user review when available.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="34" customHeight="1" s="92">
       <c r="A49" s="99" t="inlineStr">
@@ -4543,7 +4548,7 @@
           <t>Not Submitted</t>
         </is>
       </c>
-      <c r="H49" s="101" t="str"/>
+      <c r="H49" s="101" t="n"/>
     </row>
     <row r="50" ht="34" customHeight="1" s="92">
       <c r="A50" s="99" t="inlineStr">

</xml_diff>

<commit_message>
T27 enforce RabbitMQ service identities
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R99d77cc51e1046b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R16c6b4ff5d034858"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R98393bc214e14109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R5c4468ac626b4c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf2158e0dca1e4273"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R411334999ddb49c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rc2c4c2d0e39749fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R52850d50cbcf42ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1226,22 +1226,18 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5 - Security &amp; Observability</x:t>
-        </x:is>
+      <x:c r="B25" s="8" t="n">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C25" s="9" t="n">
-        <x:f>COUNTIF('Tasks'!$B$2:$B$999,B25)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D25" s="9" t="n">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="D25" s="9" t="n">
-        <x:f>COUNTIFS('Tasks'!$B$2:$B$999,B25,'Tasks'!$G$2:$G$999,"Completed")</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="E25" s="9" t="n">
         <x:f>C25-D25</x:f>
-        <x:v>4</x:v>
+        <x:v>-3</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1287,10 +1283,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="C28" s="11" t="n">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
         <x:v>12</x:v>
@@ -2341,10 +2337,8 @@
           <x:t xml:space="preserve">T07, T14</x:t>
         </x:is>
       </x:c>
-      <x:c r="G28" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G28" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="29" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2804,7 +2798,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82dd10ce29ca4d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbec70e9aac524898"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4551,15 +4545,14 @@
         </x:is>
       </x:c>
       <x:c r="F50" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A50,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G50" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H50" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G50" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H50" s="101" t="str">
+        <x:v>Implemented: RabbitMQ connection options now bind existing HostName/UserName keys, reject blank/shared default broker credentials, expose TLS settings, apply service identity/TLS to the RabbitMQ client factory, and document concrete workload identities.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A51" s="99" t="inlineStr">
@@ -4950,8 +4943,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d30444ee39641dc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b2905501b7e4cdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b50e080529f4062"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf33e29f893e643e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T28 allowlist RabbitMQ forwarded telemetry headers
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf2158e0dca1e4273"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R411334999ddb49c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rc2c4c2d0e39749fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R52850d50cbcf42ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4e9e21ce2112446e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R12f9d8970b804742"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R2890f88515ad4580"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R4cfb170242404e02"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1212,32 +1212,31 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="B24" s="8" t="n">
-        <x:v>5</x:v>
+      <x:c r="B24" s="8" t="str">
+        <x:v>4 - Downstream &amp; Deletion</x:v>
       </x:c>
       <x:c r="C24" s="9" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="D24" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E24" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="B25" s="8" t="n">
-        <x:v>5</x:v>
+      <x:c r="B25" s="8" t="str">
+        <x:v>5 - Security &amp; Observability</x:v>
       </x:c>
       <x:c r="C25" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D25" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E25" s="9" t="n">
-        <x:f>C25-D25</x:f>
-        <x:v>-3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1279,17 +1278,17 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="B28" s="10" t="n">
+      <x:c r="B28" s="10" t="str">
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="C28" s="11" t="n">
-        <x:v>27</x:v>
-      </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2372,10 +2371,8 @@
           <x:t xml:space="preserve">T17, T18, T22, T27</x:t>
         </x:is>
       </x:c>
-      <x:c r="G29" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G29" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="30" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2798,7 +2795,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbec70e9aac524898"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1126537801d45c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4581,15 +4578,14 @@
         </x:is>
       </x:c>
       <x:c r="F51" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A51,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G51" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H51" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G51" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H51" s="101" t="str">
+        <x:v>Implemented: RabbitMQ retry/DLQ header forwarding now uses an allowlist for trace context plus retry attempt, with canary tests proving filenames, blob paths, transcript previews, provider bodies, and authorization secrets do not persist as broker headers.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A52" s="99" t="inlineStr">
@@ -4943,8 +4939,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b50e080529f4062"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf33e29f893e643e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0afbbb97f13448fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R497528992d624b5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T29 add event bus health and safe metrics
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4e9e21ce2112446e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R12f9d8970b804742"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R2890f88515ad4580"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R4cfb170242404e02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc0f41286718f41f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rae1e6fe5ea3e481e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R827b47809c3e44e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R9c53800394094516"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1233,10 +1233,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D25" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E25" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1285,10 +1285,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2406,10 +2406,8 @@
           <x:t xml:space="preserve">T11, T20, T22, T25, T28</x:t>
         </x:is>
       </x:c>
-      <x:c r="G30" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G30" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="31" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2795,7 +2793,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1126537801d45c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd34deada0d74aa9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4614,15 +4612,14 @@
         </x:is>
       </x:c>
       <x:c r="F52" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A52,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G52" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H52" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G52" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H52" s="101" t="str">
+        <x:v>Implemented: backend health/live and health/ready endpoints, reusable RabbitMQ subscriber readiness checks, worker readiness reuse, RabbitMQ delivery metrics, and outbox relay metrics with safe dimensions only.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A53" s="99" t="inlineStr">
@@ -4939,8 +4936,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0afbbb97f13448fb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R497528992d624b5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb50ac585711e4865"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04adb1ee91f04366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T30 enforce event replay and retention policy
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc0f41286718f41f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rae1e6fe5ea3e481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R827b47809c3e44e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R9c53800394094516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R241fd4d632f94429"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R401bcd8b03744370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R9b68cf8a04464340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Re8d26ed30b3d4a1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1233,10 +1233,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D25" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E25" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1285,10 +1285,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2441,10 +2441,8 @@
           <x:t xml:space="preserve">T20, T25, T27, T28</x:t>
         </x:is>
       </x:c>
-      <x:c r="G31" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G31" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="32" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2793,7 +2791,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd34deada0d74aa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3063190b5574d17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4648,15 +4646,14 @@
         </x:is>
       </x:c>
       <x:c r="F53" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A53,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G53" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H53" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G53" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H53" s="101" t="str">
+        <x:v>Implemented: replay policy requires immutable original event ID, operator identity, and reason; rejects replacement payload JSON; adds EventRetention options/validation requiring tombstones to outlive event records; documents runbook controls.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A54" s="99" t="inlineStr">
@@ -4936,8 +4933,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb50ac585711e4865"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04adb1ee91f04366"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R187934076eba4e3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ae132fd6af14273"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T31 add containerized local stack
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R241fd4d632f94429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R401bcd8b03744370"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R9b68cf8a04464340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Re8d26ed30b3d4a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3d67f280c3df43d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R9403422ce4754b2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rb5397edd63c24107"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rf76eadb1a0b54557"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1240,22 +1240,17 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="B26" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6 - Containers &amp; Operations</x:t>
-        </x:is>
+      <x:c r="B26" s="8" t="str">
+        <x:v>6 - Containers &amp; Operations</x:v>
       </x:c>
       <x:c r="C26" s="9" t="n">
-        <x:f>COUNTIF('Tasks'!$B$2:$B$999,B26)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D26" s="9" t="n">
-        <x:f>COUNTIFS('Tasks'!$B$2:$B$999,B26,'Tasks'!$G$2:$G$999,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E26" s="9" t="n">
-        <x:f>C26-D26</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1285,10 +1280,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2476,10 +2471,8 @@
           <x:t xml:space="preserve">T14, T22, T27</x:t>
         </x:is>
       </x:c>
-      <x:c r="G32" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G32" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="33" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2791,7 +2784,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3063190b5574d17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb161c107fd7e490a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4682,15 +4675,14 @@
         </x:is>
       </x:c>
       <x:c r="F54" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A54,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G54" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H54" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G54" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H54" s="101" t="str">
+        <x:v>Implemented: Dockerfiles for backend API, migrations, Transcription Worker, and Clinical Knowledge API; root Compose stack with PostgreSQL, pgvector PostgreSQL, RabbitMQ provisioning, Azurite, health checks, migrations, API, worker, and Clinical Knowledge services; compose env example.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A55" s="99" t="inlineStr">
@@ -4933,8 +4925,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R187934076eba4e3b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ae132fd6af14273"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a3d9d0f32de4630"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra48f8c569c9648bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T32 validate scaling and deployment controls
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3d67f280c3df43d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R9403422ce4754b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rb5397edd63c24107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rf76eadb1a0b54557"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd24e76e493a64a0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rbb8419739597463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rf1bde9d5804148d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rd54f0d5557974e73"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1247,10 +1247,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D26" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E26" s="9" t="n">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="E26" s="9" t="n">
-        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1280,10 +1280,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2506,10 +2506,8 @@
           <x:t xml:space="preserve">T21, T29, T31</x:t>
         </x:is>
       </x:c>
-      <x:c r="G33" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G33" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="34" s="92" customFormat="1" ht="87" customHeight="1">
@@ -2784,7 +2782,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb161c107fd7e490a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5cdf6b6303e4d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4711,15 +4709,14 @@
         </x:is>
       </x:c>
       <x:c r="F55" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A55,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G55" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H55" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G55" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H55" s="101" t="str">
+        <x:v>Implemented: validated worker concurrency/prefetch, shutdown drain, processing lease, RabbitMQ consumer settings, and outbox relay batch/lease/poll/backoff limits; exposed Compose scaling variables; documented scaling and expand-contract tuning behavior.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A56" s="99" t="inlineStr">
@@ -4925,8 +4922,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a3d9d0f32de4630"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra48f8c569c9648bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R525f4d23605648fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c27d6aad4748fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T33 add guarded DLQ replay seam
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd24e76e493a64a0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rbb8419739597463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rf1bde9d5804148d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rd54f0d5557974e73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7391607cd91940df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rb22c520dbf1c44b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R8b5ddee2d7fd4db9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R397b165f0cf6405e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1247,10 +1247,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D26" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E26" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1280,10 +1280,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2541,10 +2541,8 @@
           <x:t xml:space="preserve">T20, T29, T30, T31</x:t>
         </x:is>
       </x:c>
-      <x:c r="G34" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G34" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="35" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2782,7 +2780,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5cdf6b6303e4d8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R858ace7ec7f94157"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4745,15 +4743,14 @@
         </x:is>
       </x:c>
       <x:c r="F56" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A56,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G56" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H56" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G56" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H56" s="101" t="str">
+        <x:v>Implemented: approved DLQ replay seam with safe metadata inspection, replay authorization, contract safety check extension, immutable envelope republish through RabbitMQ publisher confirms, PHI-safe audit/result details, and operations runbook updates.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A57" s="99" t="inlineStr">
@@ -4922,8 +4919,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R525f4d23605648fe"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c27d6aad4748fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f5b48bf4d4e4acb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf919dd3a97b84bf7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T34 add executable failure matrix
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7391607cd91940df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rb22c520dbf1c44b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R8b5ddee2d7fd4db9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="R397b165f0cf6405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb7ab98396ea14701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R438b537ab7504052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R8f3f701d0c0f4437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Raa0abe1c52eb4b3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1254,22 +1254,17 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="B27" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">7 - Verification &amp; Removal</x:t>
-        </x:is>
+      <x:c r="B27" s="8" t="str">
+        <x:v>7 - Verification &amp; Removal</x:v>
       </x:c>
       <x:c r="C27" s="9" t="n">
-        <x:f>COUNTIF('Tasks'!$B$2:$B$999,B27)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D27" s="9" t="n">
-        <x:f>COUNTIFS('Tasks'!$B$2:$B$999,B27,'Tasks'!$G$2:$G$999,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E27" s="9" t="n">
-        <x:f>C27-D27</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1280,10 +1275,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2576,10 +2571,8 @@
           <x:t xml:space="preserve">T31, T32, T33</x:t>
         </x:is>
       </x:c>
-      <x:c r="G35" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G35" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="36" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2780,7 +2773,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R858ace7ec7f94157"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda1e6614f1194062"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4779,15 +4772,14 @@
         </x:is>
       </x:c>
       <x:c r="F57" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A57,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G57" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H57" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G57" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H57" s="101" t="str">
+        <x:v>Implemented: living end-to-end failure matrix documentation for all 12 root-Compose scenarios plus executable coverage tests that verify each scenario has automated backend evidence and no placeholder outcomes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A58" s="99" t="inlineStr">
@@ -4919,8 +4911,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f5b48bf4d4e4acb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf919dd3a97b84bf7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d16df63cb2b4131"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63218f58d4094c23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T35 enforce architecture and privacy guardrails
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb7ab98396ea14701"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R438b537ab7504052"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R8f3f701d0c0f4437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Raa0abe1c52eb4b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2528799207ca4f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rbe42304fe9bd4edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rb150776096cf4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Re711335b8a3c4877"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1261,10 +1261,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D27" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E27" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1275,10 +1275,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2606,10 +2606,8 @@
           <x:t xml:space="preserve">T28, T34</x:t>
         </x:is>
       </x:c>
-      <x:c r="G36" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G36" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="37" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2773,7 +2771,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda1e6614f1194062"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f70a339aedc4578"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4808,15 +4806,14 @@
         </x:is>
       </x:c>
       <x:c r="F58" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A58,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G58" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H58" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G58" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H58" s="101" t="str">
+        <x:v>Implemented: removed obsolete Azure Function transcriber and legacy direct RabbitMQ publisher code/config; added active source/config enforcement tests for Functions artifacts, legacy queues, default-exchange publishing, reflection routing, automatic host migrations, queue-draining APIs, and PHI telemetry canaries.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A59" s="99" t="inlineStr">
@@ -4911,8 +4908,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d16df63cb2b4131"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63218f58d4094c23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ba367bed1aa457d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca4b87f2b6f4cfb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T36 verify legacy removal completion
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2528799207ca4f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Rbe42304fe9bd4edb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="Rb150776096cf4be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Re711335b8a3c4877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra3efd29ef2ca4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Ra76d5e2f8a5c4271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R4163e8ddeef64bc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rf5e72800b4894238"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1261,10 +1261,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D27" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E27" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1275,10 +1275,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2641,10 +2641,8 @@
           <x:t xml:space="preserve">T34, T35</x:t>
         </x:is>
       </x:c>
-      <x:c r="G37" s="73" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G37" s="73" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="38" s="92" customFormat="1" ht="72" customHeight="1">
@@ -2771,7 +2769,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f70a339aedc4578"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R525eddfa79ea401b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4842,15 +4840,14 @@
         </x:is>
       </x:c>
       <x:c r="F59" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A59,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G59" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H59" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G59" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H59" s="101" t="str">
+        <x:v>Implemented: added an explicit legacy-removal verification record and executable tests proving the Azure Function transcriber, direct RabbitMQ publisher paths, legacy queue settings, and duplicate removal behaviors are gone while the standalone worker keeps the useful Blob/Speech seams.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" s="92" customFormat="1" ht="34" customHeight="1">
       <x:c r="A60" s="99" t="inlineStr">
@@ -4908,8 +4905,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ba367bed1aa457d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca4b87f2b6f4cfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfe8971b867644ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9002dc065b574735"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
T37 add clean environment release gate
</commit_message>
<xml_diff>
--- a/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
+++ b/project-docs/event bus implementations/event-bus-implementation-tasks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra3efd29ef2ca4542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="Ra76d5e2f8a5c4271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R4163e8ddeef64bc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rf5e72800b4894238"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9ee70a0589df4728"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R029cbc3e3f9041ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Bugs" sheetId="3" r:id="R69f53fda4ddb411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Plan" sheetId="4" r:id="Rf1581ccbe2fc411f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1261,10 +1261,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D27" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E27" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1275,10 +1275,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2676,10 +2676,8 @@
           <x:t xml:space="preserve">T36</x:t>
         </x:is>
       </x:c>
-      <x:c r="G38" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Started</x:t>
-        </x:is>
+      <x:c r="G38" s="70" t="str">
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2769,7 +2767,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R525eddfa79ea401b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf1eac57088d46b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4876,15 +4874,14 @@
         </x:is>
       </x:c>
       <x:c r="F60" s="95" t="str">
-        <x:f>INDEX('Tasks'!$G$2:$G$38,MATCH(A60,'Tasks'!$A$2:$A$38,0))</x:f>
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="G60" s="101" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not Submitted</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H60" s="101" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="G60" s="101" t="str">
+        <x:v>Review Deferred</x:v>
+      </x:c>
+      <x:c r="H60" s="101" t="str">
+        <x:v>Implemented: added the clean-environment release gate with stop-release policy, Compose/migration/test/no-Functions commands, release evidence template, security and operations review, dashboard/alert coverage, backup/restore rehearsal, and executable documentation guardrails.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4905,8 +4902,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfe8971b867644ec"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9002dc065b574735"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37c41d9317364bcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6e5817cc46d4bf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>